<commit_message>
Confirm 9019 10 10 00 for LN Shop Nails pedicure spa chairs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DgQWpMLzULgi9Px8QXRVhU
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_LN_Shop_Nails_XME26080221.xlsx
+++ b/output/HS_Code_Summary_LN_Shop_Nails_XME26080221.xlsx
@@ -46,7 +46,7 @@
       <color rgb="00C00000"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -56,11 +56,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,9 +118,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -500,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -618,7 +610,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>9019 10 10 00 (ověřit)</t>
+          <t>9019 10 10 00 (potvrzeno)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -658,14 +650,10 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>OVĚŘIT ZAŘAZENÍ</t>
-        </is>
-      </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>HS dle B/L (shipper). Nejednoznačné: 9019 10 (masážní přístroj) vs. 9402 10 00 (holičská/pedikérská a podobná křesla). Křesla (8728-CHAIR) + podstavce (S842/S858-BASE) = 45 kompletních křesel v rozloženém stavu (VPV 2a). 8728-LEATHER, KM AUTOFILL a Magnet jet jsou náhradní díly/příslušenství – na faktuře BEZ popisu, B/L je zahrnuje do pol. 1 (149 balíků). Případně konzultovat s customs.tariff@mauriceward.com.</t>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>HS dle B/L (shipper) – POTVRZENO: 9019 10 10 00 použito u předchozích zásilek LN Shop Nails („Elektrické vibrační masážní přístroje – elektrické pedikér…“). Křesla (8728-CHAIR) + podstavce (S842/S858-BASE) = 45 kompletních křesel v rozloženém stavu (VPV 2a). 8728-LEATHER, KM AUTOFILL a Magnet jet = náhradní díly/příslušenství, zahrnuty s křeslem dle B/L (pol. 1, 149 balíků).</t>
         </is>
       </c>
     </row>
@@ -722,12 +710,12 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>OPRAVA KN</t>
         </is>
       </c>
-      <c r="N6" s="9" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Kód 9403200000 není platný 10místný TARIC (9403 20 se v KN dělí na 20 = lůžka / 80 = ostatní). Mycí lůžko není lůžko ke spaní → 9403 20 80 (ostatní kovový nábytek), pokud je kostra kovová. Ověřit materiál.</t>
         </is>
@@ -786,12 +774,12 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>OPRAVA KN</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>Kód 3926909090 v KN neexistuje (3926 90 se dělí na 50 / 92 / 97). Plastový vzorník laků na nehty → 3926 90 97. Pokud by šlo o tištěný papírový vzorník, zvážit kap. 49 – ověřit.</t>
         </is>
@@ -850,12 +838,12 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="M8" s="10" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>CBAM + MELT&amp;POUR</t>
         </is>
       </c>
-      <c r="N8" s="10" t="inlineStr">
+      <c r="N8" s="9" t="inlineStr">
         <is>
           <t>Kód 7326909000 v KN neexistuje (7326 90 se dělí na 30/40/50/60/92/94/96/98) → 7326 90 98 (ostatní výrobky ze železa/oceli). CBAM zboží (č. 7326). Příjemce LN SHOP NAILS NENÍ v CBAM registru! Chybí hutní atest (melt &amp; pour).</t>
         </is>
@@ -922,44 +910,44 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="11" t="inlineStr">
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>209 balíků</t>
         </is>
       </c>
-      <c r="H10" s="12" t="n"/>
-      <c r="I10" s="13">
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="12">
         <f>SUM(I5:I9)</f>
         <v/>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="12">
         <f>SUM(J5:J9)</f>
         <v/>
       </c>
-      <c r="K10" s="14">
+      <c r="K10" s="13">
         <f>SUM(K5:K9)</f>
         <v/>
       </c>
-      <c r="L10" s="12" t="n"/>
-      <c r="M10" s="12" t="n"/>
-      <c r="N10" s="15" t="inlineStr">
+      <c r="L10" s="11" t="n"/>
+      <c r="M10" s="11" t="n"/>
+      <c r="N10" s="14" t="inlineStr">
         <is>
           <t>Kontrola: NW 7 497,5 kg (PL zaokr. 7 498) | GW 8 220 kg (= PL i B/L) | Total faktury USD 48 600,00</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Legenda:</t>
         </is>
@@ -967,7 +955,7 @@
       <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>🔴 ČERVENÁ</t>
         </is>
@@ -979,48 +967,36 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>🟠 ORANŽOVÁ</t>
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>🟡 ŽLUTÁ</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sazební zařazení nejednoznačné – ověřit (případně tarifní tým)</t>
+          <t>HS kód odesílatele není platný v KN/TARIC EU – navržena oprava 8místného kódu (CCT/VPV KN tariff rule)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>🟡 ŽLUTÁ</t>
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Hodnota</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HS kód odesílatele není platný v KN/TARIC EU – navržena oprava 8místného kódu (CCT/VPV KN tariff rule)</t>
+          <t>Částky z obchodní faktury KM260429-2, celková částka 'TOTAL: $48,600.00'. Bez slevy.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Hodnota</t>
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Hmotnosti</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
-        <is>
-          <t>Částky z obchodní faktury KM260429-2, celková částka 'TOTAL: $48,600.00'. Bez slevy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Hmotnosti</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
         <is>
           <t>Skutečné NW/GW z packing listu (ne proporcionální výpočet). GW souhlasí s B/L po skupinách.</t>
         </is>
@@ -1044,7 +1020,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16">
+      <c r="A1" s="15">
         <f>== PŘIJATÉ DOKUMENTY ===</f>
         <v/>
       </c>
@@ -1088,7 +1064,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="16">
+      <c r="A8" s="15">
         <f>== ODESÍLATEL / TŘÍDĚNÍ ===</f>
         <v/>
       </c>
@@ -1104,20 +1080,20 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16">
+      <c r="A11" s="15">
         <f>== POPIS ZBOŽÍ ===</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>⚠ Klient NEZASLAL český popis zboží. Ve sloupci Popis je anglický popis z obchodní faktury. Sloupec 'Orientační CZ překlad' je můj překlad, nikoli popis od klienta – před podáním potvrdit s klientem.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>⚠ Na faktuře nemají popis ani model řádky 15 ks (USD 45) a 10 ks (USD 20) – dle packing listu jde o 'KM AUTOFILL' a 'Magnet jet'. Doporučeno vyžádat popis/funkci.</t>
         </is>
@@ -1127,7 +1103,7 @@
       <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="16">
+      <c r="A15" s="15">
         <f>== INCOTERM / CELNÍ HODNOTA ===</f>
         <v/>
       </c>
@@ -1140,7 +1116,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>⚠ ROZPOR: B/L uvádí FREIGHT COLLECT a Euro/Shipping fakturuje kupujícímu námořní dopravné z FOB YANTIAN (ocean freight 4 750 USD). Při CFR by dopravné hradil prodávající.</t>
         </is>
@@ -1161,14 +1137,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>⚠ Pozn.: Bremerhaven ≠ Hamburg (místo CFR na faktuře). Potvrdit s klientem skutečnou dodací podmínku.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>⚠ Faktura Euro-Shipping 2026103 uvádí kontejner MRSU264738-0 – NESOUHLASÍ s MRKU4536490 (potvrzení Euro/Shipping uvádí správně MRKU453649-0). Vyžádat opravu faktury.</t>
         </is>
@@ -1223,7 +1199,7 @@
       <c r="A29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="16">
+      <c r="A30" s="15">
         <f>== PREFERENČNÍ PŮVOD / COO ===</f>
         <v/>
       </c>
@@ -1236,14 +1212,14 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>✗ Preferenční věta (prohlášení o preferenčním původu) NENÍ v dokladech uvedena → platí standardní (smluvní) clo třetích zemí. EU nemá s Čínou preferenční dohodu.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>✗ REX číslo NENÍ na faktuře uvedeno.</t>
         </is>
@@ -1253,7 +1229,7 @@
       <c r="A34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="16">
+      <c r="A35" s="15">
         <f>== CBAM ===</f>
         <v/>
       </c>
@@ -1266,7 +1242,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>⚠ Příjemce LN SHOP NAILS S.R.O. (IČO 14170191, EORI/DIČ CZ14170191) NENÍ v registru reference/CBAM_receivers_CZ.xlsx (hledáno dle firmy i EORI).</t>
         </is>
@@ -1290,13 +1266,13 @@
       <c r="A40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="16">
+      <c r="A41" s="15">
         <f>== MELT AND POUR (ocel) ===</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>⚠ Pro položku 7326 (nerezový stojan na plakáty) CHYBÍ hutní atest / mill test certificate a země tavby a odlití (melt &amp; pour). Nutno vyžádat před proclením.</t>
         </is>
@@ -1313,7 +1289,7 @@
       <c r="A44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="16">
+      <c r="A45" s="15">
         <f>== ANTIDUMPING ===</f>
         <v/>
       </c>
@@ -1329,7 +1305,7 @@
       <c r="A47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="16">
+      <c r="A48" s="15">
         <f>== SAZEBNÍ ZAŘAZENÍ (CCT/VPV KN tariff rule) ===</f>
         <v/>
       </c>
@@ -1351,14 +1327,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>9019101000 (pedikérské křeslo): kód je platný, ale zařazení je sporné – alternativa 9402 10 00 (holičská, zubařská a podobná křesla). Rozhoduje, zda podstatný charakter dává masážní funkce, nebo křeslo.</t>
+          <t>9019101000 (pedikérské křeslo): POTVRZENO – 9019 10 10 00 použito u předchozích zásilek LN Shop Nails (alternativa 9402 10 00 se neuplatní).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Pro T1 postačuje 6místný HS kód – kódy odesílatele na 6 místech jsou použitelné, kromě sporu 9019/9402.</t>
+          <t>Pro T1 postačuje 6místný HS kód – kódy odesílatele na 6 místech jsou použitelné, u 3926 / 7326 / 9403 doporučeno uvést opravený 8místný KN.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spa chair code: based on previous shipments, electric function not evidenced in docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DgQWpMLzULgi9Px8QXRVhU
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_LN_Shop_Nails_XME26080221.xlsx
+++ b/output/HS_Code_Summary_LN_Shop_Nails_XME26080221.xlsx
@@ -610,7 +610,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>9019 10 10 00 (potvrzeno)</t>
+          <t>9019 10 10 00 (dle předchozích zásilek)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -653,7 +653,7 @@
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>HS dle B/L (shipper) – POTVRZENO: 9019 10 10 00 použito u předchozích zásilek LN Shop Nails („Elektrické vibrační masážní přístroje – elektrické pedikér…“). Křesla (8728-CHAIR) + podstavce (S842/S858-BASE) = 45 kompletních křesel v rozloženém stavu (VPV 2a). 8728-LEATHER, KM AUTOFILL a Magnet jet = náhradní díly/příslušenství, zahrnuty s křeslem dle B/L (pol. 1, 149 balíků).</t>
+          <t>HS dle B/L (shipper); 9019 10 10 00 použito i u předchozích zásilek LN Shop Nails („Elektrické vibrační masážní přístroje – elektrické pedikér…“). ⚠ V dokladech této zásilky NENÍ uvedeno, že jde o elektrický vibrační masážní přístroj – pokud by nebyl elektrický/vibrační → 9019 10 90. Doporučeno vyžádat technický list / foto štítku (napětí, příkon, masážní mechanismus). Křesla (8728-CHAIR) + podstavce (S842/S858-BASE) = 45 kompletních křesel v rozloženém stavu (VPV 2a). 8728-LEATHER, KM AUTOFILL a Magnet jet = náhradní díly/příslušenství, zahrnuty s křeslem dle B/L (pol. 1, 149 balíků).</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>9019101000 (pedikérské křeslo): POTVRZENO – 9019 10 10 00 použito u předchozích zásilek LN Shop Nails (alternativa 9402 10 00 se neuplatní).</t>
+          <t>9019101000 (pedikérské křeslo): 9019 10 10 00 dle kódu odesílatele a předchozích zásilek LN Shop Nails. Elektrická vibrační masáž NENÍ v dokladech této zásilky doložena – ověřit technickým listem (jinak 9019 10 90).</t>
         </is>
       </c>
     </row>

</xml_diff>